<commit_message>
Actualizacion de plantillas de Excel para Revaluacion
</commit_message>
<xml_diff>
--- a/doc/REVALUACIÓN DE PROVEEDORES.xlsx
+++ b/doc/REVALUACIÓN DE PROVEEDORES.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\JURIDICA - CONTRATACION PS\2024\REVALUACION DE PROVEDORES\SEGUNDO CONTRATO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Soporte y Desarrollo\Documents\NetBeansProjects\combinacion\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{614B47D8-8DE6-4447-ACEE-E77678525532}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="4080" windowHeight="6432"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EVALUACION" sheetId="1" r:id="rId1"/>
@@ -20,7 +21,7 @@
     <definedName name="OLE_LINK1" localSheetId="0">#REF!</definedName>
     <definedName name="Z_F9937E7B_518C_4447_9917_3D07A617439F_.wvu.PrintTitles" localSheetId="0">EVALUACION!$1:$12</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="PaS51oB9cU5ptAtwz/Yghy0CMcmRIMND+PE9/BuoiFY="/>
@@ -338,7 +339,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;\ #,##0"/>
   </numFmts>
@@ -752,8 +753,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+  <cellXfs count="67">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -779,9 +780,6 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -801,16 +799,16 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -819,62 +817,30 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -886,22 +852,20 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -909,6 +873,40 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -938,12 +936,18 @@
     <xdr:ext cx="8343900" cy="1219200"/>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="2" name="Shape 2"/>
+        <xdr:cNvPr id="2" name="Shape 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGrpSpPr/>
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="234950" y="0"/>
+          <a:off x="228600" y="0"/>
           <a:ext cx="8343900" cy="1219200"/>
           <a:chOff x="1174050" y="3170400"/>
           <a:chExt cx="8343900" cy="1219200"/>
@@ -951,7 +955,13 @@
       </xdr:grpSpPr>
       <xdr:grpSp>
         <xdr:nvGrpSpPr>
-          <xdr:cNvPr id="3" name="Shape 3"/>
+          <xdr:cNvPr id="3" name="Shape 3">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
           <xdr:cNvGrpSpPr/>
         </xdr:nvGrpSpPr>
         <xdr:grpSpPr>
@@ -964,7 +974,13 @@
         </xdr:grpSpPr>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="4" name="Shape 4"/>
+            <xdr:cNvPr id="4" name="Shape 4">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
             <xdr:cNvSpPr/>
           </xdr:nvSpPr>
           <xdr:spPr>
@@ -1001,7 +1017,13 @@
         </xdr:sp>
         <xdr:grpSp>
           <xdr:nvGrpSpPr>
-            <xdr:cNvPr id="5" name="Shape 5"/>
+            <xdr:cNvPr id="5" name="Shape 5">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
             <xdr:cNvGrpSpPr/>
           </xdr:nvGrpSpPr>
           <xdr:grpSpPr>
@@ -1014,7 +1036,13 @@
           </xdr:grpSpPr>
           <xdr:sp macro="" textlink="">
             <xdr:nvSpPr>
-              <xdr:cNvPr id="6" name="Shape 6"/>
+              <xdr:cNvPr id="6" name="Shape 6">
+                <a:extLst>
+                  <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000006000000}"/>
+                  </a:ext>
+                </a:extLst>
+              </xdr:cNvPr>
               <xdr:cNvSpPr/>
             </xdr:nvSpPr>
             <xdr:spPr>
@@ -1053,7 +1081,13 @@
           </xdr:sp>
           <xdr:grpSp>
             <xdr:nvGrpSpPr>
-              <xdr:cNvPr id="7" name="Shape 7"/>
+              <xdr:cNvPr id="7" name="Shape 7">
+                <a:extLst>
+                  <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000007000000}"/>
+                  </a:ext>
+                </a:extLst>
+              </xdr:cNvPr>
               <xdr:cNvGrpSpPr/>
             </xdr:nvGrpSpPr>
             <xdr:grpSpPr>
@@ -1066,7 +1100,13 @@
             </xdr:grpSpPr>
             <xdr:sp macro="" textlink="">
               <xdr:nvSpPr>
-                <xdr:cNvPr id="8" name="Shape 8"/>
+                <xdr:cNvPr id="8" name="Shape 8">
+                  <a:extLst>
+                    <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                      <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000008000000}"/>
+                    </a:ext>
+                  </a:extLst>
+                </xdr:cNvPr>
                 <xdr:cNvSpPr/>
               </xdr:nvSpPr>
               <xdr:spPr>
@@ -1111,7 +1151,13 @@
             </xdr:sp>
             <xdr:sp macro="" textlink="">
               <xdr:nvSpPr>
-                <xdr:cNvPr id="9" name="Shape 9"/>
+                <xdr:cNvPr id="9" name="Shape 9">
+                  <a:extLst>
+                    <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                      <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000009000000}"/>
+                    </a:ext>
+                  </a:extLst>
+                </xdr:cNvPr>
                 <xdr:cNvSpPr txBox="1"/>
               </xdr:nvSpPr>
               <xdr:spPr>
@@ -1175,7 +1221,13 @@
             </xdr:sp>
             <xdr:sp macro="" textlink="">
               <xdr:nvSpPr>
-                <xdr:cNvPr id="10" name="Shape 10"/>
+                <xdr:cNvPr id="10" name="Shape 10">
+                  <a:extLst>
+                    <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                      <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000A000000}"/>
+                    </a:ext>
+                  </a:extLst>
+                </xdr:cNvPr>
                 <xdr:cNvSpPr/>
               </xdr:nvSpPr>
               <xdr:spPr>
@@ -1241,7 +1293,13 @@
             </xdr:sp>
             <xdr:sp macro="" textlink="">
               <xdr:nvSpPr>
-                <xdr:cNvPr id="11" name="Shape 11"/>
+                <xdr:cNvPr id="11" name="Shape 11">
+                  <a:extLst>
+                    <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                      <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000B000000}"/>
+                    </a:ext>
+                  </a:extLst>
+                </xdr:cNvPr>
                 <xdr:cNvSpPr/>
               </xdr:nvSpPr>
               <xdr:spPr>
@@ -1303,7 +1361,13 @@
             </xdr:sp>
             <xdr:sp macro="" textlink="">
               <xdr:nvSpPr>
-                <xdr:cNvPr id="12" name="Shape 12"/>
+                <xdr:cNvPr id="12" name="Shape 12">
+                  <a:extLst>
+                    <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                      <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000C000000}"/>
+                    </a:ext>
+                  </a:extLst>
+                </xdr:cNvPr>
                 <xdr:cNvSpPr txBox="1"/>
               </xdr:nvSpPr>
               <xdr:spPr>
@@ -1484,7 +1548,13 @@
           </xdr:grpSp>
           <xdr:pic>
             <xdr:nvPicPr>
-              <xdr:cNvPr id="13" name="Shape 13" descr="escudo"/>
+              <xdr:cNvPr id="13" name="Shape 13" descr="escudo">
+                <a:extLst>
+                  <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000D000000}"/>
+                  </a:ext>
+                </a:extLst>
+              </xdr:cNvPr>
               <xdr:cNvPicPr preferRelativeResize="0"/>
             </xdr:nvPicPr>
             <xdr:blipFill rotWithShape="1">
@@ -1523,7 +1593,13 @@
     <xdr:ext cx="2152650" cy="314325"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="14" name="Shape 14"/>
+        <xdr:cNvPr id="14" name="Shape 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000E000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -1806,25 +1882,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:AA995"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.59765625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="2.796875" customWidth="1"/>
-    <col min="2" max="2" width="3.59765625" customWidth="1"/>
-    <col min="3" max="3" width="16.69921875" customWidth="1"/>
-    <col min="4" max="5" width="12.3984375" customWidth="1"/>
+    <col min="1" max="1" width="2.75" customWidth="1"/>
+    <col min="2" max="2" width="3.625" customWidth="1"/>
+    <col min="3" max="3" width="16.75" customWidth="1"/>
+    <col min="4" max="5" width="12.375" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="12.3984375" customWidth="1"/>
-    <col min="8" max="8" width="11.69921875" customWidth="1"/>
-    <col min="9" max="9" width="10.59765625" customWidth="1"/>
-    <col min="10" max="10" width="12.3984375" customWidth="1"/>
-    <col min="11" max="11" width="8.09765625" customWidth="1"/>
-    <col min="12" max="12" width="2.09765625" customWidth="1"/>
-    <col min="13" max="27" width="9.3984375" customWidth="1"/>
+    <col min="7" max="7" width="12.375" customWidth="1"/>
+    <col min="8" max="8" width="11.75" customWidth="1"/>
+    <col min="9" max="9" width="10.625" customWidth="1"/>
+    <col min="10" max="10" width="12.375" customWidth="1"/>
+    <col min="11" max="11" width="8.125" customWidth="1"/>
+    <col min="12" max="12" width="2.125" customWidth="1"/>
+    <col min="13" max="27" width="9.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:27" ht="14.4">
+    <row r="1" spans="2:27">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -1836,7 +1912,7 @@
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
     </row>
-    <row r="2" spans="2:27" ht="14.4">
+    <row r="2" spans="2:27">
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -1860,7 +1936,7 @@
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
     </row>
-    <row r="4" spans="2:27" ht="14.4">
+    <row r="4" spans="2:27">
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -1872,7 +1948,7 @@
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
     </row>
-    <row r="5" spans="2:27" ht="14.4">
+    <row r="5" spans="2:27">
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -1884,7 +1960,7 @@
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
     </row>
-    <row r="6" spans="2:27" ht="14.4">
+    <row r="6" spans="2:27">
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
@@ -1909,34 +1985,34 @@
       <c r="K7" s="1"/>
     </row>
     <row r="8" spans="2:27" ht="22.5" customHeight="1">
-      <c r="B8" s="27" t="s">
+      <c r="B8" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="C8" s="28"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="28"/>
-      <c r="I8" s="28"/>
-      <c r="J8" s="28"/>
-      <c r="K8" s="29"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+      <c r="I8" s="27"/>
+      <c r="J8" s="27"/>
+      <c r="K8" s="28"/>
     </row>
     <row r="9" spans="2:27" ht="30" customHeight="1">
-      <c r="B9" s="31" t="s">
+      <c r="B9" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="C9" s="29"/>
-      <c r="D9" s="32" t="s">
+      <c r="C9" s="28"/>
+      <c r="D9" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="28"/>
-      <c r="I9" s="28"/>
-      <c r="J9" s="28"/>
-      <c r="K9" s="29"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="27"/>
+      <c r="J9" s="27"/>
+      <c r="K9" s="28"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
       <c r="N9" s="1"/>
@@ -1955,20 +2031,20 @@
       <c r="AA9" s="1"/>
     </row>
     <row r="10" spans="2:27" ht="30" customHeight="1">
-      <c r="B10" s="31" t="s">
+      <c r="B10" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="29"/>
-      <c r="D10" s="27" t="s">
+      <c r="C10" s="28"/>
+      <c r="D10" s="30" t="s">
         <v>61</v>
       </c>
-      <c r="E10" s="66"/>
-      <c r="F10" s="66"/>
-      <c r="G10" s="66"/>
-      <c r="H10" s="66"/>
-      <c r="I10" s="66"/>
-      <c r="J10" s="66"/>
-      <c r="K10" s="67"/>
+      <c r="E10" s="47"/>
+      <c r="F10" s="47"/>
+      <c r="G10" s="47"/>
+      <c r="H10" s="47"/>
+      <c r="I10" s="47"/>
+      <c r="J10" s="47"/>
+      <c r="K10" s="48"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
       <c r="N10" s="1"/>
@@ -1987,19 +2063,19 @@
       <c r="AA10" s="1"/>
     </row>
     <row r="11" spans="2:27" ht="22.5" customHeight="1">
-      <c r="B11" s="35" t="s">
+      <c r="B11" s="49" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="36"/>
-      <c r="D11" s="35" t="s">
+      <c r="C11" s="51"/>
+      <c r="D11" s="49" t="s">
         <v>75</v>
       </c>
       <c r="E11" s="50"/>
-      <c r="F11" s="36"/>
-      <c r="G11" s="52" t="s">
+      <c r="F11" s="51"/>
+      <c r="G11" s="54" t="s">
         <v>6</v>
       </c>
-      <c r="H11" s="36"/>
+      <c r="H11" s="51"/>
       <c r="I11" s="3" t="s">
         <v>7</v>
       </c>
@@ -2027,13 +2103,13 @@
       <c r="AA11" s="1"/>
     </row>
     <row r="12" spans="2:27" ht="28.5" customHeight="1">
-      <c r="B12" s="37"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="37"/>
-      <c r="E12" s="51"/>
-      <c r="F12" s="38"/>
-      <c r="G12" s="37"/>
-      <c r="H12" s="38"/>
+      <c r="B12" s="52"/>
+      <c r="C12" s="53"/>
+      <c r="D12" s="52"/>
+      <c r="E12" s="40"/>
+      <c r="F12" s="53"/>
+      <c r="G12" s="52"/>
+      <c r="H12" s="53"/>
       <c r="I12" s="6">
         <v>6</v>
       </c>
@@ -2061,20 +2137,20 @@
       <c r="AA12" s="1"/>
     </row>
     <row r="13" spans="2:27" ht="30" customHeight="1">
-      <c r="B13" s="39" t="s">
+      <c r="B13" s="62" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="34"/>
-      <c r="D13" s="45" t="s">
+      <c r="C13" s="56"/>
+      <c r="D13" s="60" t="s">
         <v>78</v>
       </c>
-      <c r="E13" s="28"/>
-      <c r="F13" s="28"/>
-      <c r="G13" s="28"/>
-      <c r="H13" s="28"/>
-      <c r="I13" s="28"/>
-      <c r="J13" s="28"/>
-      <c r="K13" s="29"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="27"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="27"/>
+      <c r="I13" s="27"/>
+      <c r="J13" s="27"/>
+      <c r="K13" s="28"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
       <c r="N13" s="1"/>
@@ -2093,20 +2169,20 @@
       <c r="AA13" s="1"/>
     </row>
     <row r="14" spans="2:27" ht="41.25" customHeight="1">
-      <c r="B14" s="32" t="s">
+      <c r="B14" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="29"/>
-      <c r="D14" s="32" t="s">
+      <c r="C14" s="28"/>
+      <c r="D14" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="E14" s="28"/>
-      <c r="F14" s="28"/>
-      <c r="G14" s="28"/>
-      <c r="H14" s="28"/>
-      <c r="I14" s="28"/>
-      <c r="J14" s="28"/>
-      <c r="K14" s="29"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="27"/>
+      <c r="I14" s="27"/>
+      <c r="J14" s="27"/>
+      <c r="K14" s="28"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
@@ -2125,20 +2201,20 @@
       <c r="AA14" s="1"/>
     </row>
     <row r="15" spans="2:27" ht="30" customHeight="1">
-      <c r="B15" s="32" t="s">
+      <c r="B15" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="29"/>
-      <c r="D15" s="32" t="s">
+      <c r="C15" s="28"/>
+      <c r="D15" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="E15" s="28"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28"/>
-      <c r="H15" s="28"/>
-      <c r="I15" s="28"/>
-      <c r="J15" s="28"/>
-      <c r="K15" s="29"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="27"/>
+      <c r="J15" s="27"/>
+      <c r="K15" s="28"/>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
@@ -2157,20 +2233,20 @@
       <c r="AA15" s="1"/>
     </row>
     <row r="16" spans="2:27" ht="30" customHeight="1">
-      <c r="B16" s="31" t="s">
+      <c r="B16" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="29"/>
-      <c r="D16" s="46" t="s">
+      <c r="C16" s="28"/>
+      <c r="D16" s="61" t="s">
         <v>16</v>
       </c>
-      <c r="E16" s="28"/>
-      <c r="F16" s="28"/>
-      <c r="G16" s="28"/>
-      <c r="H16" s="28"/>
-      <c r="I16" s="28"/>
-      <c r="J16" s="28"/>
-      <c r="K16" s="29"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="27"/>
+      <c r="I16" s="27"/>
+      <c r="J16" s="27"/>
+      <c r="K16" s="28"/>
       <c r="L16" s="1"/>
       <c r="M16" s="1"/>
       <c r="N16" s="1"/>
@@ -2189,20 +2265,20 @@
       <c r="AA16" s="1"/>
     </row>
     <row r="17" spans="2:11" ht="30" customHeight="1">
-      <c r="B17" s="32" t="s">
+      <c r="B17" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="29"/>
-      <c r="D17" s="46" t="s">
+      <c r="C17" s="28"/>
+      <c r="D17" s="61" t="s">
         <v>74</v>
       </c>
-      <c r="E17" s="28"/>
-      <c r="F17" s="28"/>
-      <c r="G17" s="28"/>
-      <c r="H17" s="28"/>
-      <c r="I17" s="28"/>
-      <c r="J17" s="28"/>
-      <c r="K17" s="29"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="27"/>
+      <c r="I17" s="27"/>
+      <c r="J17" s="27"/>
+      <c r="K17" s="28"/>
     </row>
     <row r="18" spans="2:11" ht="4.5" customHeight="1">
       <c r="B18" s="1"/>
@@ -2217,51 +2293,51 @@
       <c r="K18" s="1"/>
     </row>
     <row r="19" spans="2:11" ht="22.5" customHeight="1">
-      <c r="B19" s="27" t="s">
+      <c r="B19" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
-      <c r="F19" s="28"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="28"/>
-      <c r="I19" s="28"/>
-      <c r="J19" s="28"/>
-      <c r="K19" s="29"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
+      <c r="I19" s="27"/>
+      <c r="J19" s="27"/>
+      <c r="K19" s="28"/>
     </row>
     <row r="20" spans="2:11" ht="30" customHeight="1">
-      <c r="B20" s="33" t="s">
+      <c r="B20" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="C20" s="34"/>
-      <c r="D20" s="33" t="s">
+      <c r="C20" s="56"/>
+      <c r="D20" s="55" t="s">
         <v>20</v>
       </c>
-      <c r="E20" s="40"/>
-      <c r="F20" s="40"/>
-      <c r="G20" s="34"/>
-      <c r="H20" s="33" t="s">
+      <c r="E20" s="64"/>
+      <c r="F20" s="64"/>
+      <c r="G20" s="56"/>
+      <c r="H20" s="55" t="s">
         <v>21</v>
       </c>
-      <c r="I20" s="34"/>
-      <c r="J20" s="33" t="s">
+      <c r="I20" s="56"/>
+      <c r="J20" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="K20" s="34"/>
+      <c r="K20" s="56"/>
     </row>
     <row r="21" spans="2:11" ht="30" customHeight="1">
-      <c r="B21" s="35" t="s">
+      <c r="B21" s="49" t="s">
         <v>23</v>
       </c>
-      <c r="C21" s="36"/>
-      <c r="D21" s="32" t="s">
+      <c r="C21" s="51"/>
+      <c r="D21" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="E21" s="28"/>
-      <c r="F21" s="28"/>
-      <c r="G21" s="29"/>
-      <c r="H21" s="43">
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="28"/>
+      <c r="H21" s="57">
         <v>60</v>
       </c>
       <c r="I21" s="6">
@@ -2270,57 +2346,57 @@
       <c r="J21" s="9">
         <v>30</v>
       </c>
-      <c r="K21" s="43">
+      <c r="K21" s="57">
         <v>60</v>
       </c>
     </row>
     <row r="22" spans="2:11" ht="30" customHeight="1">
-      <c r="B22" s="41"/>
-      <c r="C22" s="42"/>
-      <c r="D22" s="32" t="s">
+      <c r="B22" s="65"/>
+      <c r="C22" s="66"/>
+      <c r="D22" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="E22" s="28"/>
-      <c r="F22" s="28"/>
-      <c r="G22" s="29"/>
-      <c r="H22" s="44"/>
+      <c r="E22" s="27"/>
+      <c r="F22" s="27"/>
+      <c r="G22" s="28"/>
+      <c r="H22" s="58"/>
       <c r="I22" s="6">
         <v>15</v>
       </c>
       <c r="J22" s="9">
         <v>15</v>
       </c>
-      <c r="K22" s="44"/>
+      <c r="K22" s="58"/>
     </row>
     <row r="23" spans="2:11" ht="30" customHeight="1">
-      <c r="B23" s="37"/>
-      <c r="C23" s="38"/>
-      <c r="D23" s="32" t="s">
+      <c r="B23" s="52"/>
+      <c r="C23" s="53"/>
+      <c r="D23" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="E23" s="28"/>
-      <c r="F23" s="28"/>
-      <c r="G23" s="29"/>
-      <c r="H23" s="53"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="28"/>
+      <c r="H23" s="59"/>
       <c r="I23" s="6">
         <v>15</v>
       </c>
       <c r="J23" s="9">
         <v>15</v>
       </c>
-      <c r="K23" s="53"/>
+      <c r="K23" s="59"/>
     </row>
     <row r="24" spans="2:11" ht="30" customHeight="1">
-      <c r="B24" s="35" t="s">
+      <c r="B24" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="36"/>
-      <c r="D24" s="32" t="s">
+      <c r="C24" s="51"/>
+      <c r="D24" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="E24" s="28"/>
-      <c r="F24" s="28"/>
-      <c r="G24" s="29"/>
+      <c r="E24" s="27"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="28"/>
       <c r="H24" s="8">
         <v>10</v>
       </c>
@@ -2330,22 +2406,22 @@
       <c r="J24" s="9">
         <v>10</v>
       </c>
-      <c r="K24" s="10">
+      <c r="K24" s="6">
         <v>10</v>
       </c>
     </row>
     <row r="25" spans="2:11" ht="30" customHeight="1">
-      <c r="B25" s="35" t="s">
+      <c r="B25" s="49" t="s">
         <v>29</v>
       </c>
-      <c r="C25" s="36"/>
-      <c r="D25" s="32" t="s">
+      <c r="C25" s="51"/>
+      <c r="D25" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="E25" s="28"/>
-      <c r="F25" s="28"/>
-      <c r="G25" s="29"/>
-      <c r="H25" s="43">
+      <c r="E25" s="27"/>
+      <c r="F25" s="27"/>
+      <c r="G25" s="28"/>
+      <c r="H25" s="57">
         <v>30</v>
       </c>
       <c r="I25" s="6">
@@ -2354,55 +2430,55 @@
       <c r="J25" s="9">
         <v>10</v>
       </c>
-      <c r="K25" s="43">
+      <c r="K25" s="57">
         <v>30</v>
       </c>
     </row>
     <row r="26" spans="2:11" ht="30" customHeight="1">
-      <c r="B26" s="41"/>
-      <c r="C26" s="42"/>
-      <c r="D26" s="32" t="s">
+      <c r="B26" s="65"/>
+      <c r="C26" s="66"/>
+      <c r="D26" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="E26" s="28"/>
-      <c r="F26" s="28"/>
-      <c r="G26" s="29"/>
-      <c r="H26" s="44"/>
+      <c r="E26" s="27"/>
+      <c r="F26" s="27"/>
+      <c r="G26" s="28"/>
+      <c r="H26" s="58"/>
       <c r="I26" s="6">
         <v>10</v>
       </c>
       <c r="J26" s="9">
         <v>10</v>
       </c>
-      <c r="K26" s="44"/>
+      <c r="K26" s="58"/>
     </row>
     <row r="27" spans="2:11" ht="42" customHeight="1">
-      <c r="B27" s="37"/>
-      <c r="C27" s="38"/>
-      <c r="D27" s="32" t="s">
+      <c r="B27" s="52"/>
+      <c r="C27" s="53"/>
+      <c r="D27" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="E27" s="28"/>
-      <c r="F27" s="28"/>
-      <c r="G27" s="29"/>
-      <c r="H27" s="44"/>
+      <c r="E27" s="27"/>
+      <c r="F27" s="27"/>
+      <c r="G27" s="28"/>
+      <c r="H27" s="58"/>
       <c r="I27" s="6">
         <v>10</v>
       </c>
       <c r="J27" s="9">
         <v>10</v>
       </c>
-      <c r="K27" s="53"/>
+      <c r="K27" s="59"/>
     </row>
     <row r="28" spans="2:11" ht="30" customHeight="1">
-      <c r="B28" s="27" t="s">
+      <c r="B28" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="C28" s="28"/>
-      <c r="D28" s="28"/>
-      <c r="E28" s="28"/>
-      <c r="F28" s="28"/>
-      <c r="G28" s="29"/>
+      <c r="C28" s="27"/>
+      <c r="D28" s="27"/>
+      <c r="E28" s="27"/>
+      <c r="F28" s="27"/>
+      <c r="G28" s="28"/>
       <c r="H28" s="6">
         <f t="shared" ref="H28:I28" si="0">SUM(H21:H27)</f>
         <v>100</v>
@@ -2411,42 +2487,42 @@
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="J28" s="27">
+      <c r="J28" s="30">
         <f>SUM(K21:K27)</f>
         <v>100</v>
       </c>
-      <c r="K28" s="29"/>
+      <c r="K28" s="28"/>
     </row>
     <row r="29" spans="2:11" ht="30" customHeight="1">
-      <c r="B29" s="27" t="s">
+      <c r="B29" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="28"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="28"/>
-      <c r="H29" s="28"/>
-      <c r="I29" s="29"/>
-      <c r="J29" s="54" t="str">
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="27"/>
+      <c r="F29" s="27"/>
+      <c r="G29" s="27"/>
+      <c r="H29" s="27"/>
+      <c r="I29" s="28"/>
+      <c r="J29" s="35" t="str">
         <f>IF(J28&lt;65,B37,IF(J28&lt;75,B36,IF(J28&lt;90,B35,B34)))</f>
         <v>Satisfactorio</v>
       </c>
-      <c r="K29" s="29"/>
+      <c r="K29" s="28"/>
     </row>
     <row r="30" spans="2:11" ht="105" customHeight="1">
-      <c r="B30" s="47" t="s">
+      <c r="B30" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="C30" s="28"/>
-      <c r="D30" s="28"/>
-      <c r="E30" s="28"/>
-      <c r="F30" s="28"/>
-      <c r="G30" s="28"/>
-      <c r="H30" s="28"/>
-      <c r="I30" s="28"/>
-      <c r="J30" s="28"/>
-      <c r="K30" s="29"/>
+      <c r="C30" s="27"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="27"/>
+      <c r="F30" s="27"/>
+      <c r="G30" s="27"/>
+      <c r="H30" s="27"/>
+      <c r="I30" s="27"/>
+      <c r="J30" s="27"/>
+      <c r="K30" s="28"/>
     </row>
     <row r="31" spans="2:11" ht="4.5" customHeight="1">
       <c r="B31" s="1"/>
@@ -2461,404 +2537,404 @@
       <c r="K31" s="1"/>
     </row>
     <row r="32" spans="2:11" ht="22.5" customHeight="1">
-      <c r="B32" s="27" t="s">
+      <c r="B32" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="28"/>
-      <c r="D32" s="28"/>
-      <c r="E32" s="28"/>
-      <c r="F32" s="28"/>
-      <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
-      <c r="I32" s="28"/>
-      <c r="J32" s="28"/>
-      <c r="K32" s="29"/>
+      <c r="C32" s="27"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="27"/>
+      <c r="F32" s="27"/>
+      <c r="G32" s="27"/>
+      <c r="H32" s="27"/>
+      <c r="I32" s="27"/>
+      <c r="J32" s="27"/>
+      <c r="K32" s="28"/>
     </row>
     <row r="33" spans="2:27" ht="30" customHeight="1">
-      <c r="B33" s="54" t="s">
+      <c r="B33" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="C33" s="29"/>
-      <c r="D33" s="54" t="s">
+      <c r="C33" s="28"/>
+      <c r="D33" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="E33" s="29"/>
-      <c r="F33" s="63" t="s">
+      <c r="E33" s="28"/>
+      <c r="F33" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="G33" s="28"/>
-      <c r="H33" s="28"/>
-      <c r="I33" s="28"/>
-      <c r="J33" s="28"/>
-      <c r="K33" s="29"/>
+      <c r="G33" s="27"/>
+      <c r="H33" s="27"/>
+      <c r="I33" s="27"/>
+      <c r="J33" s="27"/>
+      <c r="K33" s="28"/>
     </row>
     <row r="34" spans="2:27" ht="52.5" customHeight="1">
-      <c r="B34" s="27" t="s">
+      <c r="B34" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="C34" s="29"/>
-      <c r="D34" s="62" t="s">
+      <c r="C34" s="28"/>
+      <c r="D34" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="E34" s="29"/>
-      <c r="F34" s="62" t="s">
+      <c r="E34" s="28"/>
+      <c r="F34" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="G34" s="28"/>
-      <c r="H34" s="28"/>
-      <c r="I34" s="28"/>
-      <c r="J34" s="28"/>
-      <c r="K34" s="29"/>
+      <c r="G34" s="27"/>
+      <c r="H34" s="27"/>
+      <c r="I34" s="27"/>
+      <c r="J34" s="27"/>
+      <c r="K34" s="28"/>
     </row>
     <row r="35" spans="2:27" ht="52.5" customHeight="1">
-      <c r="B35" s="27" t="s">
+      <c r="B35" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="C35" s="29"/>
-      <c r="D35" s="62" t="s">
+      <c r="C35" s="28"/>
+      <c r="D35" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="E35" s="29"/>
-      <c r="F35" s="62" t="s">
+      <c r="E35" s="28"/>
+      <c r="F35" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="G35" s="28"/>
-      <c r="H35" s="28"/>
-      <c r="I35" s="28"/>
-      <c r="J35" s="28"/>
-      <c r="K35" s="29"/>
+      <c r="G35" s="27"/>
+      <c r="H35" s="27"/>
+      <c r="I35" s="27"/>
+      <c r="J35" s="27"/>
+      <c r="K35" s="28"/>
     </row>
     <row r="36" spans="2:27" ht="52.5" customHeight="1">
-      <c r="B36" s="27" t="s">
+      <c r="B36" s="30" t="s">
         <v>45</v>
       </c>
-      <c r="C36" s="29"/>
-      <c r="D36" s="62" t="s">
+      <c r="C36" s="28"/>
+      <c r="D36" s="32" t="s">
         <v>46</v>
       </c>
-      <c r="E36" s="29"/>
-      <c r="F36" s="62" t="s">
+      <c r="E36" s="28"/>
+      <c r="F36" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="G36" s="28"/>
-      <c r="H36" s="28"/>
-      <c r="I36" s="28"/>
-      <c r="J36" s="28"/>
-      <c r="K36" s="29"/>
+      <c r="G36" s="27"/>
+      <c r="H36" s="27"/>
+      <c r="I36" s="27"/>
+      <c r="J36" s="27"/>
+      <c r="K36" s="28"/>
     </row>
     <row r="37" spans="2:27" ht="52.5" customHeight="1">
-      <c r="B37" s="27" t="s">
+      <c r="B37" s="30" t="s">
         <v>48</v>
       </c>
-      <c r="C37" s="29"/>
-      <c r="D37" s="27" t="s">
+      <c r="C37" s="28"/>
+      <c r="D37" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="E37" s="29"/>
-      <c r="F37" s="62" t="s">
+      <c r="E37" s="28"/>
+      <c r="F37" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="G37" s="28"/>
-      <c r="H37" s="28"/>
-      <c r="I37" s="28"/>
-      <c r="J37" s="28"/>
-      <c r="K37" s="29"/>
+      <c r="G37" s="27"/>
+      <c r="H37" s="27"/>
+      <c r="I37" s="27"/>
+      <c r="J37" s="27"/>
+      <c r="K37" s="28"/>
     </row>
     <row r="38" spans="2:27" ht="4.5" customHeight="1">
-      <c r="B38" s="48"/>
-      <c r="C38" s="49"/>
+      <c r="B38" s="33"/>
+      <c r="C38" s="34"/>
       <c r="D38" s="1"/>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
       <c r="G38" s="1"/>
-      <c r="H38" s="48"/>
-      <c r="I38" s="49"/>
-      <c r="J38" s="49"/>
-      <c r="K38" s="49"/>
+      <c r="H38" s="33"/>
+      <c r="I38" s="34"/>
+      <c r="J38" s="34"/>
+      <c r="K38" s="34"/>
     </row>
     <row r="39" spans="2:27" ht="22.5" customHeight="1">
-      <c r="B39" s="27" t="s">
+      <c r="B39" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="C39" s="28"/>
-      <c r="D39" s="28"/>
-      <c r="E39" s="28"/>
-      <c r="F39" s="28"/>
-      <c r="G39" s="28"/>
-      <c r="H39" s="28"/>
-      <c r="I39" s="28"/>
-      <c r="J39" s="28"/>
-      <c r="K39" s="29"/>
+      <c r="C39" s="27"/>
+      <c r="D39" s="27"/>
+      <c r="E39" s="27"/>
+      <c r="F39" s="27"/>
+      <c r="G39" s="27"/>
+      <c r="H39" s="27"/>
+      <c r="I39" s="27"/>
+      <c r="J39" s="27"/>
+      <c r="K39" s="28"/>
     </row>
     <row r="40" spans="2:27" ht="22.5" customHeight="1">
-      <c r="B40" s="30" t="s">
+      <c r="B40" s="63" t="s">
         <v>52</v>
       </c>
-      <c r="C40" s="28"/>
-      <c r="D40" s="28"/>
-      <c r="E40" s="28"/>
-      <c r="F40" s="28"/>
-      <c r="G40" s="28"/>
-      <c r="H40" s="28"/>
-      <c r="I40" s="28"/>
-      <c r="J40" s="28"/>
-      <c r="K40" s="29"/>
-      <c r="L40" s="11"/>
-      <c r="M40" s="11"/>
-      <c r="N40" s="11"/>
-      <c r="O40" s="11"/>
-      <c r="P40" s="11"/>
-      <c r="Q40" s="11"/>
-      <c r="R40" s="11"/>
-      <c r="S40" s="11"/>
-      <c r="T40" s="11"/>
-      <c r="U40" s="11"/>
-      <c r="V40" s="11"/>
-      <c r="W40" s="11"/>
-      <c r="X40" s="11"/>
-      <c r="Y40" s="11"/>
-      <c r="Z40" s="11"/>
-      <c r="AA40" s="11"/>
+      <c r="C40" s="27"/>
+      <c r="D40" s="27"/>
+      <c r="E40" s="27"/>
+      <c r="F40" s="27"/>
+      <c r="G40" s="27"/>
+      <c r="H40" s="27"/>
+      <c r="I40" s="27"/>
+      <c r="J40" s="27"/>
+      <c r="K40" s="28"/>
+      <c r="L40" s="10"/>
+      <c r="M40" s="10"/>
+      <c r="N40" s="10"/>
+      <c r="O40" s="10"/>
+      <c r="P40" s="10"/>
+      <c r="Q40" s="10"/>
+      <c r="R40" s="10"/>
+      <c r="S40" s="10"/>
+      <c r="T40" s="10"/>
+      <c r="U40" s="10"/>
+      <c r="V40" s="10"/>
+      <c r="W40" s="10"/>
+      <c r="X40" s="10"/>
+      <c r="Y40" s="10"/>
+      <c r="Z40" s="10"/>
+      <c r="AA40" s="10"/>
     </row>
     <row r="41" spans="2:27" ht="25.5" customHeight="1">
       <c r="B41" s="6"/>
-      <c r="C41" s="31" t="s">
+      <c r="C41" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="D41" s="28"/>
-      <c r="E41" s="28"/>
-      <c r="F41" s="28"/>
-      <c r="G41" s="28"/>
-      <c r="H41" s="28"/>
-      <c r="I41" s="28"/>
-      <c r="J41" s="28"/>
-      <c r="K41" s="29"/>
+      <c r="D41" s="27"/>
+      <c r="E41" s="27"/>
+      <c r="F41" s="27"/>
+      <c r="G41" s="27"/>
+      <c r="H41" s="27"/>
+      <c r="I41" s="27"/>
+      <c r="J41" s="27"/>
+      <c r="K41" s="28"/>
     </row>
     <row r="42" spans="2:27" ht="25.5" customHeight="1">
       <c r="B42" s="6"/>
-      <c r="C42" s="31" t="s">
+      <c r="C42" s="46" t="s">
         <v>54</v>
       </c>
-      <c r="D42" s="28"/>
-      <c r="E42" s="28"/>
-      <c r="F42" s="28"/>
-      <c r="G42" s="28"/>
-      <c r="H42" s="28"/>
-      <c r="I42" s="28"/>
-      <c r="J42" s="28"/>
-      <c r="K42" s="29"/>
+      <c r="D42" s="27"/>
+      <c r="E42" s="27"/>
+      <c r="F42" s="27"/>
+      <c r="G42" s="27"/>
+      <c r="H42" s="27"/>
+      <c r="I42" s="27"/>
+      <c r="J42" s="27"/>
+      <c r="K42" s="28"/>
     </row>
     <row r="43" spans="2:27" ht="25.5" customHeight="1">
       <c r="B43" s="6"/>
-      <c r="C43" s="31" t="s">
+      <c r="C43" s="46" t="s">
         <v>55</v>
       </c>
-      <c r="D43" s="28"/>
-      <c r="E43" s="28"/>
-      <c r="F43" s="28"/>
-      <c r="G43" s="28"/>
-      <c r="H43" s="28"/>
-      <c r="I43" s="28"/>
-      <c r="J43" s="28"/>
-      <c r="K43" s="29"/>
+      <c r="D43" s="27"/>
+      <c r="E43" s="27"/>
+      <c r="F43" s="27"/>
+      <c r="G43" s="27"/>
+      <c r="H43" s="27"/>
+      <c r="I43" s="27"/>
+      <c r="J43" s="27"/>
+      <c r="K43" s="28"/>
     </row>
     <row r="44" spans="2:27" ht="25.5" customHeight="1">
       <c r="B44" s="6"/>
-      <c r="C44" s="31" t="s">
+      <c r="C44" s="46" t="s">
         <v>56</v>
       </c>
-      <c r="D44" s="28"/>
-      <c r="E44" s="28"/>
-      <c r="F44" s="28"/>
-      <c r="G44" s="28"/>
-      <c r="H44" s="28"/>
-      <c r="I44" s="28"/>
-      <c r="J44" s="28"/>
-      <c r="K44" s="29"/>
+      <c r="D44" s="27"/>
+      <c r="E44" s="27"/>
+      <c r="F44" s="27"/>
+      <c r="G44" s="27"/>
+      <c r="H44" s="27"/>
+      <c r="I44" s="27"/>
+      <c r="J44" s="27"/>
+      <c r="K44" s="28"/>
     </row>
     <row r="45" spans="2:27" ht="25.5" customHeight="1">
       <c r="B45" s="6"/>
-      <c r="C45" s="31" t="s">
+      <c r="C45" s="46" t="s">
         <v>57</v>
       </c>
-      <c r="D45" s="28"/>
-      <c r="E45" s="28"/>
-      <c r="F45" s="28"/>
-      <c r="G45" s="28"/>
-      <c r="H45" s="28"/>
-      <c r="I45" s="28"/>
-      <c r="J45" s="28"/>
-      <c r="K45" s="29"/>
+      <c r="D45" s="27"/>
+      <c r="E45" s="27"/>
+      <c r="F45" s="27"/>
+      <c r="G45" s="27"/>
+      <c r="H45" s="27"/>
+      <c r="I45" s="27"/>
+      <c r="J45" s="27"/>
+      <c r="K45" s="28"/>
     </row>
     <row r="46" spans="2:27" ht="25.5" customHeight="1">
       <c r="B46" s="6"/>
-      <c r="C46" s="31" t="s">
+      <c r="C46" s="46" t="s">
         <v>58</v>
       </c>
-      <c r="D46" s="28"/>
-      <c r="E46" s="28"/>
-      <c r="F46" s="28"/>
-      <c r="G46" s="28"/>
-      <c r="H46" s="28"/>
-      <c r="I46" s="28"/>
-      <c r="J46" s="28"/>
-      <c r="K46" s="29"/>
+      <c r="D46" s="27"/>
+      <c r="E46" s="27"/>
+      <c r="F46" s="27"/>
+      <c r="G46" s="27"/>
+      <c r="H46" s="27"/>
+      <c r="I46" s="27"/>
+      <c r="J46" s="27"/>
+      <c r="K46" s="28"/>
     </row>
     <row r="47" spans="2:27" ht="89.25" customHeight="1">
       <c r="B47" s="6"/>
-      <c r="C47" s="47" t="s">
+      <c r="C47" s="31" t="s">
         <v>59</v>
       </c>
-      <c r="D47" s="28"/>
-      <c r="E47" s="28"/>
-      <c r="F47" s="28"/>
-      <c r="G47" s="28"/>
-      <c r="H47" s="28"/>
-      <c r="I47" s="28"/>
-      <c r="J47" s="28"/>
-      <c r="K47" s="29"/>
+      <c r="D47" s="27"/>
+      <c r="E47" s="27"/>
+      <c r="F47" s="27"/>
+      <c r="G47" s="27"/>
+      <c r="H47" s="27"/>
+      <c r="I47" s="27"/>
+      <c r="J47" s="27"/>
+      <c r="K47" s="28"/>
     </row>
     <row r="48" spans="2:27" ht="4.5" customHeight="1">
-      <c r="B48" s="48"/>
-      <c r="C48" s="49"/>
+      <c r="B48" s="33"/>
+      <c r="C48" s="34"/>
       <c r="D48" s="1"/>
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
       <c r="G48" s="1"/>
-      <c r="H48" s="48"/>
-      <c r="I48" s="49"/>
-      <c r="J48" s="49"/>
-      <c r="K48" s="49"/>
+      <c r="H48" s="33"/>
+      <c r="I48" s="34"/>
+      <c r="J48" s="34"/>
+      <c r="K48" s="34"/>
     </row>
     <row r="49" spans="2:27" ht="22.5" customHeight="1">
-      <c r="B49" s="55" t="s">
+      <c r="B49" s="36" t="s">
         <v>60</v>
       </c>
-      <c r="C49" s="56"/>
-      <c r="D49" s="56"/>
-      <c r="E49" s="56"/>
-      <c r="F49" s="56"/>
-      <c r="G49" s="56"/>
-      <c r="H49" s="56"/>
-      <c r="I49" s="56"/>
-      <c r="J49" s="56"/>
-      <c r="K49" s="57"/>
+      <c r="C49" s="37"/>
+      <c r="D49" s="37"/>
+      <c r="E49" s="37"/>
+      <c r="F49" s="37"/>
+      <c r="G49" s="37"/>
+      <c r="H49" s="37"/>
+      <c r="I49" s="37"/>
+      <c r="J49" s="37"/>
+      <c r="K49" s="38"/>
     </row>
     <row r="50" spans="2:27" ht="18" customHeight="1">
-      <c r="B50" s="16"/>
-      <c r="C50" s="17"/>
-      <c r="D50" s="17"/>
-      <c r="E50" s="17"/>
-      <c r="F50" s="17"/>
-      <c r="G50" s="17"/>
-      <c r="H50" s="17"/>
-      <c r="I50" s="17"/>
-      <c r="J50" s="17"/>
-      <c r="K50" s="18"/>
-    </row>
-    <row r="51" spans="2:27" ht="14.4">
-      <c r="B51" s="19"/>
-      <c r="C51" s="20"/>
-      <c r="D51" s="20"/>
-      <c r="E51" s="20"/>
-      <c r="F51" s="20"/>
-      <c r="G51" s="20"/>
-      <c r="H51" s="20"/>
-      <c r="I51" s="20"/>
-      <c r="J51" s="20"/>
-      <c r="K51" s="21"/>
+      <c r="B50" s="15"/>
+      <c r="C50" s="16"/>
+      <c r="D50" s="16"/>
+      <c r="E50" s="16"/>
+      <c r="F50" s="16"/>
+      <c r="G50" s="16"/>
+      <c r="H50" s="16"/>
+      <c r="I50" s="16"/>
+      <c r="J50" s="16"/>
+      <c r="K50" s="17"/>
+    </row>
+    <row r="51" spans="2:27">
+      <c r="B51" s="18"/>
+      <c r="C51" s="19"/>
+      <c r="D51" s="19"/>
+      <c r="E51" s="19"/>
+      <c r="F51" s="19"/>
+      <c r="G51" s="19"/>
+      <c r="H51" s="19"/>
+      <c r="I51" s="19"/>
+      <c r="J51" s="19"/>
+      <c r="K51" s="20"/>
     </row>
     <row r="52" spans="2:27" ht="42" customHeight="1">
-      <c r="B52" s="58"/>
-      <c r="C52" s="51"/>
-      <c r="D52" s="51"/>
-      <c r="E52" s="51"/>
-      <c r="F52" s="22"/>
-      <c r="G52" s="23"/>
-      <c r="H52" s="23"/>
-      <c r="I52" s="23"/>
-      <c r="J52" s="23"/>
-      <c r="K52" s="24"/>
-    </row>
-    <row r="53" spans="2:27" ht="41.4" customHeight="1">
-      <c r="B53" s="64" t="s">
+      <c r="B52" s="39"/>
+      <c r="C52" s="40"/>
+      <c r="D52" s="40"/>
+      <c r="E52" s="40"/>
+      <c r="F52" s="21"/>
+      <c r="G52" s="22"/>
+      <c r="H52" s="22"/>
+      <c r="I52" s="22"/>
+      <c r="J52" s="22"/>
+      <c r="K52" s="23"/>
+    </row>
+    <row r="53" spans="2:27" ht="41.45" customHeight="1">
+      <c r="B53" s="41" t="s">
         <v>77</v>
       </c>
-      <c r="C53" s="65"/>
-      <c r="D53" s="65"/>
-      <c r="E53" s="65"/>
-      <c r="F53" s="22"/>
-      <c r="G53" s="23"/>
-      <c r="H53" s="23"/>
-      <c r="I53" s="23"/>
-      <c r="J53" s="23"/>
-      <c r="K53" s="24"/>
+      <c r="C53" s="42"/>
+      <c r="D53" s="42"/>
+      <c r="E53" s="42"/>
+      <c r="F53" s="21"/>
+      <c r="G53" s="22"/>
+      <c r="H53" s="22"/>
+      <c r="I53" s="22"/>
+      <c r="J53" s="22"/>
+      <c r="K53" s="23"/>
     </row>
     <row r="54" spans="2:27" ht="22.5" customHeight="1">
-      <c r="B54" s="25"/>
-      <c r="C54" s="26"/>
-      <c r="D54" s="23"/>
-      <c r="E54" s="22"/>
-      <c r="F54" s="22"/>
-      <c r="G54" s="23"/>
-      <c r="H54" s="23"/>
-      <c r="I54" s="23"/>
-      <c r="J54" s="23"/>
-      <c r="K54" s="24"/>
-      <c r="L54" s="11"/>
-      <c r="M54" s="11"/>
-      <c r="N54" s="11"/>
-      <c r="O54" s="11"/>
-      <c r="P54" s="11"/>
-      <c r="Q54" s="11"/>
-      <c r="R54" s="11"/>
-      <c r="S54" s="11"/>
-      <c r="T54" s="11"/>
-      <c r="U54" s="11"/>
-      <c r="V54" s="11"/>
-      <c r="W54" s="11"/>
-      <c r="X54" s="11"/>
-      <c r="Y54" s="11"/>
-      <c r="Z54" s="11"/>
-      <c r="AA54" s="11"/>
+      <c r="B54" s="24"/>
+      <c r="C54" s="25"/>
+      <c r="D54" s="22"/>
+      <c r="E54" s="21"/>
+      <c r="F54" s="21"/>
+      <c r="G54" s="22"/>
+      <c r="H54" s="22"/>
+      <c r="I54" s="22"/>
+      <c r="J54" s="22"/>
+      <c r="K54" s="23"/>
+      <c r="L54" s="10"/>
+      <c r="M54" s="10"/>
+      <c r="N54" s="10"/>
+      <c r="O54" s="10"/>
+      <c r="P54" s="10"/>
+      <c r="Q54" s="10"/>
+      <c r="R54" s="10"/>
+      <c r="S54" s="10"/>
+      <c r="T54" s="10"/>
+      <c r="U54" s="10"/>
+      <c r="V54" s="10"/>
+      <c r="W54" s="10"/>
+      <c r="X54" s="10"/>
+      <c r="Y54" s="10"/>
+      <c r="Z54" s="10"/>
+      <c r="AA54" s="10"/>
     </row>
     <row r="55" spans="2:27" ht="22.5" customHeight="1">
-      <c r="B55" s="59" t="s">
+      <c r="B55" s="43" t="s">
         <v>76</v>
       </c>
-      <c r="C55" s="60"/>
-      <c r="D55" s="60"/>
-      <c r="E55" s="60"/>
-      <c r="F55" s="60"/>
-      <c r="G55" s="60"/>
-      <c r="H55" s="60"/>
-      <c r="I55" s="60"/>
-      <c r="J55" s="60"/>
-      <c r="K55" s="61"/>
+      <c r="C55" s="44"/>
+      <c r="D55" s="44"/>
+      <c r="E55" s="44"/>
+      <c r="F55" s="44"/>
+      <c r="G55" s="44"/>
+      <c r="H55" s="44"/>
+      <c r="I55" s="44"/>
+      <c r="J55" s="44"/>
+      <c r="K55" s="45"/>
     </row>
     <row r="56" spans="2:27" ht="6.75" customHeight="1">
-      <c r="B56" s="12"/>
-      <c r="C56" s="13"/>
-      <c r="D56" s="13"/>
-      <c r="E56" s="13"/>
-      <c r="F56" s="13"/>
-      <c r="G56" s="13"/>
-      <c r="H56" s="13"/>
-      <c r="I56" s="13"/>
-      <c r="J56" s="13"/>
-      <c r="K56" s="13"/>
+      <c r="B56" s="11"/>
+      <c r="C56" s="12"/>
+      <c r="D56" s="12"/>
+      <c r="E56" s="12"/>
+      <c r="F56" s="12"/>
+      <c r="G56" s="12"/>
+      <c r="H56" s="12"/>
+      <c r="I56" s="12"/>
+      <c r="J56" s="12"/>
+      <c r="K56" s="12"/>
     </row>
     <row r="57" spans="2:27" ht="15.75" customHeight="1">
-      <c r="B57" s="14"/>
-      <c r="C57" s="14"/>
-      <c r="D57" s="14"/>
-      <c r="E57" s="14"/>
-      <c r="F57" s="14"/>
-      <c r="G57" s="14"/>
-      <c r="H57" s="14"/>
-      <c r="I57" s="14"/>
-      <c r="J57" s="14"/>
-      <c r="K57" s="14"/>
+      <c r="B57" s="13"/>
+      <c r="C57" s="13"/>
+      <c r="D57" s="13"/>
+      <c r="E57" s="13"/>
+      <c r="F57" s="13"/>
+      <c r="G57" s="13"/>
+      <c r="H57" s="13"/>
+      <c r="I57" s="13"/>
+      <c r="J57" s="13"/>
+      <c r="K57" s="13"/>
     </row>
     <row r="58" spans="2:27" ht="15.75" customHeight="1">
       <c r="B58" s="1"/>
@@ -3877,12 +3953,59 @@
     <row r="995" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="75">
-    <mergeCell ref="F33:K33"/>
-    <mergeCell ref="D27:G27"/>
-    <mergeCell ref="B28:G28"/>
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B30:K30"/>
-    <mergeCell ref="B32:K32"/>
+    <mergeCell ref="B39:K39"/>
+    <mergeCell ref="B40:K40"/>
+    <mergeCell ref="C41:K41"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="D21:G21"/>
+    <mergeCell ref="D22:G22"/>
+    <mergeCell ref="D23:G23"/>
+    <mergeCell ref="B19:K19"/>
+    <mergeCell ref="D20:G20"/>
+    <mergeCell ref="B21:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C27"/>
+    <mergeCell ref="D24:G24"/>
+    <mergeCell ref="D25:G25"/>
+    <mergeCell ref="H25:H27"/>
+    <mergeCell ref="B11:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D26:G26"/>
+    <mergeCell ref="D13:K13"/>
+    <mergeCell ref="D14:K14"/>
+    <mergeCell ref="D15:K15"/>
+    <mergeCell ref="D16:K16"/>
+    <mergeCell ref="D17:K17"/>
+    <mergeCell ref="C47:K47"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B8:K8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:K9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:K10"/>
+    <mergeCell ref="D11:F12"/>
+    <mergeCell ref="G11:H12"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="H21:H23"/>
+    <mergeCell ref="K21:K23"/>
+    <mergeCell ref="K25:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="C42:K42"/>
+    <mergeCell ref="C43:K43"/>
+    <mergeCell ref="C44:K44"/>
+    <mergeCell ref="C45:K45"/>
+    <mergeCell ref="C46:K46"/>
+    <mergeCell ref="H48:K48"/>
+    <mergeCell ref="B49:K49"/>
+    <mergeCell ref="B52:E52"/>
+    <mergeCell ref="B53:E53"/>
+    <mergeCell ref="B55:K55"/>
     <mergeCell ref="F37:K37"/>
     <mergeCell ref="H38:K38"/>
     <mergeCell ref="B33:C33"/>
@@ -3899,59 +4022,12 @@
     <mergeCell ref="F34:K34"/>
     <mergeCell ref="F35:K35"/>
     <mergeCell ref="D33:E33"/>
-    <mergeCell ref="H48:K48"/>
-    <mergeCell ref="B49:K49"/>
-    <mergeCell ref="B52:E52"/>
-    <mergeCell ref="B53:E53"/>
-    <mergeCell ref="B55:K55"/>
-    <mergeCell ref="C42:K42"/>
-    <mergeCell ref="C43:K43"/>
-    <mergeCell ref="C44:K44"/>
-    <mergeCell ref="C45:K45"/>
-    <mergeCell ref="C46:K46"/>
-    <mergeCell ref="C47:K47"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="B8:K8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D9:K9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D10:K10"/>
-    <mergeCell ref="D11:F12"/>
-    <mergeCell ref="G11:H12"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="H21:H23"/>
-    <mergeCell ref="K21:K23"/>
-    <mergeCell ref="K25:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="D26:G26"/>
-    <mergeCell ref="D13:K13"/>
-    <mergeCell ref="D14:K14"/>
-    <mergeCell ref="D15:K15"/>
-    <mergeCell ref="D16:K16"/>
-    <mergeCell ref="D17:K17"/>
-    <mergeCell ref="B11:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B39:K39"/>
-    <mergeCell ref="B40:K40"/>
-    <mergeCell ref="C41:K41"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="D21:G21"/>
-    <mergeCell ref="D22:G22"/>
-    <mergeCell ref="D23:G23"/>
-    <mergeCell ref="B19:K19"/>
-    <mergeCell ref="D20:G20"/>
-    <mergeCell ref="B21:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C27"/>
-    <mergeCell ref="D24:G24"/>
-    <mergeCell ref="D25:G25"/>
-    <mergeCell ref="H25:H27"/>
+    <mergeCell ref="F33:K33"/>
+    <mergeCell ref="D27:G27"/>
+    <mergeCell ref="B28:G28"/>
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B30:K30"/>
+    <mergeCell ref="B32:K32"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.78740157480314965" bottom="0.78740157480314965" header="0" footer="0"/>
@@ -3963,25 +4039,25 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">
-        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1">
+        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000000000000}">
           <x14:formula1>
             <xm:f>Hoja1!$H$1:$H$14</xm:f>
           </x14:formula1>
           <xm:sqref>D10</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1">
+        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000001000000}">
           <x14:formula1>
             <xm:f>Hoja1!$B$1:$B$2</xm:f>
           </x14:formula1>
           <xm:sqref>J22:J23</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1">
+        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>Hoja1!$A$1:$A$2</xm:f>
           </x14:formula1>
           <xm:sqref>J21</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1">
+        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000003000000}">
           <x14:formula1>
             <xm:f>Hoja1!$C$1:$C$2</xm:f>
           </x14:formula1>
@@ -3994,16 +4070,16 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.59765625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="7" width="9.3984375" customWidth="1"/>
-    <col min="8" max="8" width="28.19921875" customWidth="1"/>
-    <col min="9" max="26" width="9.3984375" customWidth="1"/>
+    <col min="1" max="7" width="9.375" customWidth="1"/>
+    <col min="8" max="8" width="28.25" customWidth="1"/>
+    <col min="9" max="26" width="9.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="14.4">
+    <row r="1" spans="1:8">
       <c r="A1" s="1">
         <v>0</v>
       </c>
@@ -4013,11 +4089,11 @@
       <c r="C1" s="1">
         <v>0</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="H1" s="14" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="14.4">
+    <row r="2" spans="1:8">
       <c r="A2" s="1">
         <v>30</v>
       </c>
@@ -4027,67 +4103,67 @@
       <c r="C2" s="1">
         <v>10</v>
       </c>
-      <c r="H2" s="15" t="s">
+      <c r="H2" s="14" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
-      <c r="H3" s="15" t="s">
+      <c r="H3" s="14" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
-      <c r="H4" s="15" t="s">
+      <c r="H4" s="14" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
-      <c r="H5" s="15" t="s">
+      <c r="H5" s="14" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
-      <c r="H6" s="15" t="s">
+      <c r="H6" s="14" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1">
-      <c r="H7" s="15" t="s">
+      <c r="H7" s="14" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1">
-      <c r="H8" s="15" t="s">
+      <c r="H8" s="14" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15" customHeight="1">
-      <c r="H9" s="15" t="s">
+      <c r="H9" s="14" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15" customHeight="1">
-      <c r="H10" s="15" t="s">
+      <c r="H10" s="14" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
-      <c r="H11" s="15" t="s">
+      <c r="H11" s="14" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
-      <c r="H12" s="15" t="s">
+      <c r="H12" s="14" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="15" customHeight="1">
-      <c r="H13" s="15" t="s">
+      <c r="H13" s="14" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1">
-      <c r="H14" s="15" t="s">
+      <c r="H14" s="14" t="s">
         <v>73</v>
       </c>
     </row>

</xml_diff>